<commit_message>
Diez opciones ya no terminan en el rótulo de la tabla del PDF
La auditoría integral del banco —la primera que compara también las
opciones contra el PDF; las pasadas anteriores cubrían enunciados y
campos— encontró diez que absorbieron la cabecera de la sub-tabla
siguiente: el candidato leía «…antes de reclamar Opción Clave». El
importador ahora salta esas cabeceras también dentro de una tabla de
opciones y avisa si un texto termina en rótulo; la V35 limpia lo
guardado, re-ejecutable y sin pisar ediciones del panel; MigracionesIT
lo asevera desde CI junto a la basura invisible. Los tres Excel salen
regenerados.

Del resto de la auditoría no salió nada: las claves de EF-4 y SJT-R
coinciden una a una con el PDF, los SEC cubren su orden completo, los
INV y DE declaran sus cuentas exactas y los 18 V tienen su tabla, su
referencia o su fórmula.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/insumos/banco-v3-coordinacion-y-supervision.xlsx
+++ b/docs/insumos/banco-v3-coordinacion-y-supervision.xlsx
@@ -2638,7 +2638,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Revisar si la instrucción y los recursos estaban dados antes de reclamar Opción Clave</t>
+          <t>Revisar si la instrucción y los recursos estaban dados antes de reclamar</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Me los reporta el responsable el mismo día Opción Valor</t>
+          <t>Me los reporta el responsable el mismo día</t>
         </is>
       </c>
       <c r="C78" s="7" t="n"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>Lo que más caro sale si no se hace Opción Valor</t>
+          <t>Lo que más caro sale si no se hace</t>
         </is>
       </c>
       <c r="C101" s="7" t="n"/>

</xml_diff>